<commit_message>
Add measurement-only hypothesis composition agreement and redraw Figure S15
Measurement-only has a successfully generated answer for only some LLMs per prompt
(CITE-seq 2, CosMx 3, Gouwens 2), so its agreement is judged among those LLMs
(04c, same rubric/judge/random-order passes as 04a; records in
data_available_models/). Figure S15 (plot_FigS15.py + data table) and the
three-condition radar (02f) now draw this measured value (2.89) instead of a
placeholder at the centre; READMEs updated.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/5_evaluation_results/ablation_conditions/2_quality_radar/radar_3conditions_datasheet.xlsx
+++ b/5_evaluation_results/ablation_conditions/2_quality_radar/radar_3conditions_datasheet.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Per_model_x_condition" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_model_balanced" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_individual_answers" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw_agreement_per_prompt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -458,7 +459,7 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Hypothesis composition agreement (plotted; measurement-only set to 0)</t>
+          <t>Hypothesis composition agreement (measurement-only: available models only)</t>
         </is>
       </c>
     </row>
@@ -543,7 +544,7 @@
         <v>7.643</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>2.889</v>
       </c>
     </row>
   </sheetData>
@@ -1350,6 +1351,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Prompt</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Measurement-only agreement (mean of 3 passes)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Models in the group</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CITE-seq CD45RA</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CosMx Ki-67</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2.667</v>
+      </c>
+      <c r="C3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Gouwens input resistance</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -1384,14 +1455,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>6-axis radar: hypothesis composition agreement of the measurement-only condition is set to 0 for plotting because it could not be computed; this is a placeholder, not a measured score.</t>
+          <t>6-axis radar, axis 6: PITCH and MLP + IG = hypothesis composition agreement across the 4 models (04a, mean of 3 prompts); measurement-only = agreement among the models with a successfully generated answer (CITE-seq GLM + Qwen, CosMx GLM + DeepSeek + Qwen, Gouwens Gemini + GLM; 04c; 3 passes per prompt, mean of 3 prompts). Smaller groups agree more easily, so this point is not strictly comparable.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Reproduce: 02a_select_answers.py, 02b_judge_quality.py --conds cond2_raw_data --out-dir ../../5_evaluation_results/ablation_conditions/2_quality_radar/scorecards/raw_pass1 (and raw_pass2), 02f_plot_radars_3conditions.py</t>
+          <t>Reproduce: 02a_select_answers.py, 02b_judge_quality.py --conds cond2_raw_data --out-dir ../../5_evaluation_results/ablation_conditions/2_quality_radar/scorecards/raw_pass1 (and raw_pass2), 04c_judge_hypothesis_composition_agreement_available_models.py, 02f_plot_radars_3conditions.py</t>
         </is>
       </c>
     </row>

</xml_diff>